<commit_message>
updated events for data hack
</commit_message>
<xml_diff>
--- a/src/data/events_template.xlsx
+++ b/src/data/events_template.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="252">
   <si>
     <t>Field</t>
   </si>
@@ -714,10 +714,22 @@
     <t>https://events.humanitix.com/meet-the-startups-susmi-x-sudata-x-sul-x-medscisoc</t>
   </si>
   <si>
-    <t>Datathon</t>
-  </si>
-  <si>
-    <t>SUDATA, COMM-STEM, SYNCS</t>
+    <t>Data-Hack</t>
+  </si>
+  <si>
+    <t>18/04/2026 to 20/04/2026</t>
+  </si>
+  <si>
+    <t>9am on 18th to 5pm on 20th</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multi-day datathon competition. Solve real-world data problems and win prizes! </t>
+  </si>
+  <si>
+    <t>SUDATA, COMM-STEM</t>
+  </si>
+  <si>
+    <t>https://events.humanitix.com/sudata-x-comms-stem-hackathon-2026</t>
   </si>
   <si>
     <t>Amstelveen Consulting Workshop</t>
@@ -763,6 +775,24 @@
   </si>
   <si>
     <t>https://docs.google.com/forms/d/e/1FAIpQLSe0fgyAoK7WviXjjQG5-B0WpO6OdeasQA5FbJU1cbfgnZAceQ/viewform</t>
+  </si>
+  <si>
+    <t>10:AM</t>
+  </si>
+  <si>
+    <t>Academic</t>
+  </si>
+  <si>
+    <t>Form a team to tackle real-world datasets to build innovative solutions to complex business problems. Extract insights, develop models, and get the opportunity to pitch your ideas in front of industry &amp; faculty judges.</t>
+  </si>
+  <si>
+    <t>SUDATA, Comm-STEM</t>
+  </si>
+  <si>
+    <t>Food provided throughout event</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSc0PpmEPPKaErDartdzL0OhFWrcmmq79hsq49oZ7CR2hDUi9A/viewform?fbclid=PAVERFWAQ9to9leHRuA2FlbQIxMABzcnRjBmFwcF9pZA8xMjQwMjQ1NzQyODc0MTQAAadqwtgGT7mqVE0qgxyPpec07vi01Z8i_ckhJkuwZor_kkiucx7tcICnCg-DEA_aem_-v1T0RahWKiznkVs0U-yVA&amp;pli=1</t>
   </si>
 </sst>
 </file>
@@ -774,7 +804,7 @@
     <numFmt numFmtId="165" formatCode="hh:mm"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="20">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -822,6 +852,12 @@
       <name val="-apple-system"/>
     </font>
     <font>
+      <u/>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
@@ -860,6 +896,20 @@
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="-apple-system"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -887,7 +937,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="33">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -933,41 +983,59 @@
     <xf borderId="0" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="12" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="13" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="17" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2785,7 +2853,9 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="26.63"/>
+    <col customWidth="1" min="1" max="1" width="35.88"/>
+    <col customWidth="1" min="2" max="2" width="21.25"/>
+    <col customWidth="1" min="3" max="3" width="23.25"/>
     <col customWidth="1" min="4" max="4" width="49.5"/>
     <col customWidth="1" min="5" max="5" width="13.88"/>
     <col customWidth="1" min="6" max="6" width="102.5"/>
@@ -3059,34 +3129,34 @@
       <c r="A10" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="B10" s="13">
-        <v>46111.0</v>
+      <c r="B10" s="15" t="s">
+        <v>226</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>35</v>
+        <v>227</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>35</v>
+        <v>222</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>142</v>
+        <v>228</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="I10" s="2" t="s">
-        <v>35</v>
+      <c r="I10" s="16" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B11" s="13">
         <v>46132.0</v>
@@ -3101,7 +3171,7 @@
         <v>15</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>71</v>
@@ -3115,7 +3185,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="B12" s="13">
         <v>46146.0</v>
@@ -3133,7 +3203,7 @@
         <v>45</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>35</v>
@@ -3173,7 +3243,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B14" s="13">
         <v>46174.0</v>
@@ -3188,7 +3258,7 @@
         <v>15</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>32</v>
@@ -3201,96 +3271,125 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="s">
-        <v>233</v>
-      </c>
-      <c r="B15" s="16">
+      <c r="A15" s="17" t="s">
+        <v>237</v>
+      </c>
+      <c r="B15" s="18">
         <v>46086.0</v>
       </c>
-      <c r="C15" s="17">
+      <c r="C15" s="19">
         <v>0.7083333333333334</v>
       </c>
-      <c r="D15" s="18" t="s">
-        <v>234</v>
-      </c>
-      <c r="E15" s="19" t="s">
+      <c r="D15" s="20" t="s">
+        <v>238</v>
+      </c>
+      <c r="E15" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="F15" s="20" t="s">
-        <v>235</v>
-      </c>
-      <c r="G15" s="19" t="s">
-        <v>236</v>
-      </c>
-      <c r="H15" s="21" t="s">
-        <v>237</v>
-      </c>
-      <c r="I15" s="22" t="s">
-        <v>238</v>
-      </c>
-      <c r="J15" s="15"/>
-      <c r="K15" s="15"/>
-      <c r="L15" s="15"/>
-      <c r="M15" s="15"/>
-      <c r="N15" s="15"/>
-      <c r="O15" s="15"/>
-      <c r="P15" s="15"/>
-      <c r="Q15" s="15"/>
-      <c r="R15" s="15"/>
-      <c r="S15" s="15"/>
-      <c r="T15" s="15"/>
-      <c r="U15" s="15"/>
-      <c r="V15" s="15"/>
-      <c r="W15" s="15"/>
-      <c r="X15" s="15"/>
-      <c r="Y15" s="15"/>
-      <c r="Z15" s="15"/>
+      <c r="F15" s="22" t="s">
+        <v>239</v>
+      </c>
+      <c r="G15" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="H15" s="23" t="s">
+        <v>241</v>
+      </c>
+      <c r="I15" s="24" t="s">
+        <v>242</v>
+      </c>
+      <c r="J15" s="17"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="17"/>
+      <c r="M15" s="17"/>
+      <c r="N15" s="17"/>
+      <c r="O15" s="17"/>
+      <c r="P15" s="17"/>
+      <c r="Q15" s="17"/>
+      <c r="R15" s="17"/>
+      <c r="S15" s="17"/>
+      <c r="T15" s="17"/>
+      <c r="U15" s="17"/>
+      <c r="V15" s="17"/>
+      <c r="W15" s="17"/>
+      <c r="X15" s="17"/>
+      <c r="Y15" s="17"/>
+      <c r="Z15" s="17"/>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="s">
-        <v>239</v>
-      </c>
-      <c r="B16" s="16">
+      <c r="A16" s="17" t="s">
+        <v>243</v>
+      </c>
+      <c r="B16" s="18">
         <v>46098.0</v>
       </c>
-      <c r="C16" s="23">
+      <c r="C16" s="25">
         <v>0.75</v>
       </c>
-      <c r="D16" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="19" t="s">
+      <c r="D16" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="F16" s="24" t="s">
+      <c r="F16" s="26" t="s">
+        <v>244</v>
+      </c>
+      <c r="G16" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="G16" s="19" t="s">
-        <v>236</v>
-      </c>
-      <c r="H16" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="I16" s="26" t="s">
-        <v>241</v>
-      </c>
-      <c r="J16" s="15"/>
-      <c r="K16" s="15"/>
-      <c r="L16" s="15"/>
-      <c r="M16" s="15"/>
-      <c r="N16" s="15"/>
-      <c r="O16" s="15"/>
-      <c r="P16" s="15"/>
-      <c r="Q16" s="15"/>
-      <c r="R16" s="15"/>
-      <c r="S16" s="15"/>
-      <c r="T16" s="15"/>
-      <c r="U16" s="15"/>
-      <c r="V16" s="15"/>
-      <c r="W16" s="15"/>
-      <c r="X16" s="15"/>
-      <c r="Y16" s="15"/>
-      <c r="Z16" s="15"/>
+      <c r="H16" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="I16" s="28" t="s">
+        <v>245</v>
+      </c>
+      <c r="J16" s="17"/>
+      <c r="K16" s="17"/>
+      <c r="L16" s="17"/>
+      <c r="M16" s="17"/>
+      <c r="N16" s="17"/>
+      <c r="O16" s="17"/>
+      <c r="P16" s="17"/>
+      <c r="Q16" s="17"/>
+      <c r="R16" s="17"/>
+      <c r="S16" s="17"/>
+      <c r="T16" s="17"/>
+      <c r="U16" s="17"/>
+      <c r="V16" s="17"/>
+      <c r="W16" s="17"/>
+      <c r="X16" s="17"/>
+      <c r="Y16" s="17"/>
+      <c r="Z16" s="17"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="s">
+        <v>225</v>
+      </c>
+      <c r="B17" s="30">
+        <v>46130.0</v>
+      </c>
+      <c r="C17" s="29" t="s">
+        <v>246</v>
+      </c>
+      <c r="D17" s="29" t="s">
+        <v>208</v>
+      </c>
+      <c r="E17" s="29" t="s">
+        <v>247</v>
+      </c>
+      <c r="F17" s="31" t="s">
+        <v>248</v>
+      </c>
+      <c r="G17" s="29" t="s">
+        <v>249</v>
+      </c>
+      <c r="H17" s="29" t="s">
+        <v>250</v>
+      </c>
+      <c r="I17" s="32" t="s">
+        <v>251</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3301,9 +3400,11 @@
     <hyperlink r:id="rId5" ref="I7"/>
     <hyperlink r:id="rId6" ref="I8"/>
     <hyperlink r:id="rId7" ref="I9"/>
-    <hyperlink r:id="rId8" ref="I15"/>
-    <hyperlink r:id="rId9" ref="I16"/>
+    <hyperlink r:id="rId8" ref="I10"/>
+    <hyperlink r:id="rId9" ref="I15"/>
+    <hyperlink r:id="rId10" ref="I16"/>
+    <hyperlink r:id="rId11" ref="I17"/>
   </hyperlinks>
-  <drawing r:id="rId10"/>
+  <drawing r:id="rId12"/>
 </worksheet>
 </file>
</xml_diff>